<commit_message>
HW: Notes for pin changed and ADC channel adjustment for USB-C integration
</commit_message>
<xml_diff>
--- a/hw/PS1-1/Admin/STM32G474 pinout.xlsx
+++ b/hw/PS1-1/Admin/STM32G474 pinout.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Daniel\ele\bat_source\hw\PS1-1\Admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA2C907-AFF7-45EF-B6EA-919F1803E820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C36FA24D-5C03-4004-9F8A-5141B9441838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" activeTab="3" xr2:uid="{21A4FC59-0757-4566-8791-AF29D3D9F0F9}"/>
+    <workbookView xWindow="4245" yWindow="4245" windowWidth="21600" windowHeight="12495" activeTab="4" xr2:uid="{21A4FC59-0757-4566-8791-AF29D3D9F0F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Functions" sheetId="3" r:id="rId1"/>
     <sheet name="Timer" sheetId="1" r:id="rId2"/>
     <sheet name="UART" sheetId="6" r:id="rId3"/>
-    <sheet name="ADC" sheetId="2" r:id="rId4"/>
-    <sheet name="Restricted GPIOs" sheetId="4" r:id="rId5"/>
-    <sheet name="GPIOs QFP100" sheetId="5" r:id="rId6"/>
+    <sheet name="ADC index B" sheetId="2" r:id="rId4"/>
+    <sheet name="ADC Index C" sheetId="7" r:id="rId5"/>
+    <sheet name="Restricted GPIOs" sheetId="4" r:id="rId6"/>
+    <sheet name="GPIOs QFP100" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="284">
   <si>
     <t>Timer overview</t>
   </si>
@@ -907,6 +909,18 @@
   </si>
   <si>
     <t>Pin changed during layouting</t>
+  </si>
+  <si>
+    <t>Change to</t>
+  </si>
+  <si>
+    <t>Change to ADC2 channel 5</t>
+  </si>
+  <si>
+    <t>Change to ADC2 channel 2/4</t>
+  </si>
+  <si>
+    <t>2/4</t>
   </si>
 </sst>
 </file>
@@ -936,7 +950,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -946,6 +960,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -977,7 +997,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -986,12 +1006,123 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="30">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2412,23 +2543,23 @@
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D2" s="6" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D2" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>27</v>
       </c>
@@ -2463,7 +2594,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>29</v>
       </c>
@@ -2492,7 +2623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
@@ -2515,7 +2646,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>32</v>
       </c>
@@ -2548,7 +2679,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>33</v>
       </c>
@@ -2577,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>126</v>
       </c>
@@ -2599,8 +2730,14 @@
       <c r="K8" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" t="s">
+        <v>280</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>34</v>
       </c>
@@ -2626,7 +2763,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
@@ -2649,8 +2786,14 @@
         <f>K8</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>280</v>
+      </c>
+      <c r="M10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>35</v>
       </c>
@@ -2673,7 +2816,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -2704,7 +2847,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>37</v>
       </c>
@@ -2735,7 +2878,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>38</v>
       </c>
@@ -2766,7 +2909,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>129</v>
       </c>
@@ -2787,7 +2930,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>135</v>
       </c>
@@ -2998,15 +3141,15 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -3205,6 +3348,9 @@
       </c>
       <c r="L29" s="4">
         <v>2</v>
+      </c>
+      <c r="M29" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -3262,6 +3408,9 @@
       <c r="L31" s="4">
         <v>1</v>
       </c>
+      <c r="M31" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
@@ -3635,13 +3784,1311 @@
     <mergeCell ref="D23:J23"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:C21">
-    <cfRule type="cellIs" dxfId="14" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="28" operator="equal">
       <formula>"Slow"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="29" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="30" operator="equal">
+      <formula>"Fast"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25:C42">
+    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+      <formula>"Slow"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="5" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="6" operator="equal">
+      <formula>"Fast"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:J14 D17:J21">
+    <cfRule type="cellIs" dxfId="23" priority="31" operator="equal">
+      <formula>"Protection"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="32" operator="equal">
+      <formula>"Feedforward"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="33" operator="equal">
+      <formula>"Control"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25:J35 D36:D37 F36:G37 J37">
+    <cfRule type="cellIs" dxfId="20" priority="25" operator="equal">
+      <formula>"Protection"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="26" operator="equal">
+      <formula>"Feedforward"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="27" operator="equal">
+      <formula>"Control"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D38:J42">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+      <formula>"Protection"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+      <formula>"Feedforward"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+      <formula>"Control"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9888A037-9548-402F-BC0E-8D4800ECF5F2}">
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D2" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="K6" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="4">
+        <f>K5</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K10" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D23" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="4">
+        <v>3</v>
+      </c>
+      <c r="E25" s="4">
+        <v>3</v>
+      </c>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4">
+        <v>3</v>
+      </c>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4">
+        <v>3</v>
+      </c>
+      <c r="K25" s="4">
+        <v>3</v>
+      </c>
+      <c r="L25" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4">
+        <v>4</v>
+      </c>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4">
+        <v>4</v>
+      </c>
+      <c r="L26" s="4">
+        <v>5</v>
+      </c>
+      <c r="M26" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="4">
+        <v>2</v>
+      </c>
+      <c r="E27" s="4">
+        <v>2</v>
+      </c>
+      <c r="F27" s="4">
+        <v>2</v>
+      </c>
+      <c r="G27" s="4">
+        <v>2</v>
+      </c>
+      <c r="H27" s="4">
+        <v>2</v>
+      </c>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4">
+        <v>2</v>
+      </c>
+      <c r="K27" s="4">
+        <v>2</v>
+      </c>
+      <c r="L27" s="4">
+        <v>2</v>
+      </c>
+      <c r="M27" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="4">
+        <v>1</v>
+      </c>
+      <c r="E28" s="4">
+        <v>1</v>
+      </c>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4">
+        <v>1</v>
+      </c>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4">
+        <v>1</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4">
+        <v>1</v>
+      </c>
+      <c r="L28" s="4">
+        <v>1</v>
+      </c>
+      <c r="M28" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4">
+        <v>2</v>
+      </c>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4">
+        <v>2</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="4">
+        <v>4</v>
+      </c>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4">
+        <v>4</v>
+      </c>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4">
+        <f>K26</f>
+        <v>4</v>
+      </c>
+      <c r="L30" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4">
+        <v>2</v>
+      </c>
+      <c r="K31" s="4">
+        <f>K29</f>
+        <v>2</v>
+      </c>
+      <c r="L31" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4">
+        <v>5</v>
+      </c>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" s="4">
+        <v>5</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="4">
+        <v>3</v>
+      </c>
+      <c r="G33" s="4">
+        <v>5</v>
+      </c>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4">
+        <v>4</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34" s="4">
+        <v>5</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F34" s="4">
+        <v>3</v>
+      </c>
+      <c r="G34" s="4">
+        <v>5</v>
+      </c>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4">
+        <v>4</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="4">
+        <v>5</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" s="4">
+        <v>3</v>
+      </c>
+      <c r="G35" s="4">
+        <v>5</v>
+      </c>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4">
+        <v>4</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="4">
+        <v>5</v>
+      </c>
+      <c r="E36" s="4">
+        <v>5</v>
+      </c>
+      <c r="F36" s="4">
+        <v>1</v>
+      </c>
+      <c r="G36" s="4">
+        <v>5</v>
+      </c>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4">
+        <v>1</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D37" s="4">
+        <v>5</v>
+      </c>
+      <c r="E37" s="4">
+        <v>5</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1</v>
+      </c>
+      <c r="G37" s="4">
+        <v>5</v>
+      </c>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4">
+        <v>1</v>
+      </c>
+      <c r="K37" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="L37" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" s="4">
+        <v>5</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F38" s="4">
+        <v>3</v>
+      </c>
+      <c r="G38" s="4">
+        <v>5</v>
+      </c>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4">
+        <v>4</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L38" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D39" s="4">
+        <v>5</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F39" s="4">
+        <v>3</v>
+      </c>
+      <c r="G39" s="4">
+        <v>5</v>
+      </c>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4">
+        <v>4</v>
+      </c>
+      <c r="K39" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L39" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D40" s="4">
+        <v>5</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F40" s="4">
+        <v>3</v>
+      </c>
+      <c r="G40" s="4">
+        <v>5</v>
+      </c>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4">
+        <v>4</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L40" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D41" s="4">
+        <v>5</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F41" s="4">
+        <v>3</v>
+      </c>
+      <c r="G41" s="4">
+        <v>5</v>
+      </c>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4">
+        <v>4</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D42" s="4">
+        <v>5</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F42" s="4">
+        <v>3</v>
+      </c>
+      <c r="G42" s="4">
+        <v>5</v>
+      </c>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4">
+        <v>4</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L42" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="D23:J23"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C4:C21">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
+      <formula>"Slow"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="12" operator="equal">
       <formula>"Fast"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3657,24 +5104,24 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4:J14 D17:J21">
-    <cfRule type="cellIs" dxfId="8" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="13" operator="equal">
       <formula>"Protection"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="14" operator="equal">
       <formula>"Feedforward"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="15" operator="equal">
       <formula>"Control"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D25:J35 D36:D37 F36:G37 J37">
-    <cfRule type="cellIs" dxfId="5" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"Protection"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
       <formula>"Feedforward"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
       <formula>"Control"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3694,7 +5141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B98EFC0-842C-4E2C-9ADD-C61BC67F662B}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3931,7 +5378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7680DADC-115D-4B61-ADB4-956569A4F367}">
   <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>